<commit_message>
added avonmouth as storage to project
</commit_message>
<xml_diff>
--- a/data/demo_data.xlsx
+++ b/data/demo_data.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,40 +451,45 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>avonmouth</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>hatfield_moor</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>hill_top_farm</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>holehouse_farm</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>holford</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>hornsea</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>humbly_grove</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>rough</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>stublach</t>
         </is>
@@ -500,27 +505,30 @@
         <v>6</v>
       </c>
       <c r="C2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D2" t="n">
         <v>1.5</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.8</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.7</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>4.5</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>5.2</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>2.1</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>5.5</v>
       </c>
     </row>
@@ -534,27 +542,30 @@
         <v>6.2</v>
       </c>
       <c r="C3" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D3" t="n">
         <v>1.6</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.8</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.7</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>4.7</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5.3</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>2.1</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>9</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>5.6</v>
       </c>
     </row>
@@ -568,27 +579,30 @@
         <v>5.8</v>
       </c>
       <c r="C4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D4" t="n">
         <v>1.5</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.7</v>
       </c>
       <c r="E4" t="n">
         <v>0.7</v>
       </c>
       <c r="F4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G4" t="n">
         <v>4.3</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>5.1</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>5.6</v>
       </c>
     </row>
@@ -602,27 +616,30 @@
         <v>5.6</v>
       </c>
       <c r="C5" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D5" t="n">
         <v>1.4</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>0.7</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.6</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>4.2</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>5</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>1.9</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>8.5</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>5.6</v>
       </c>
     </row>
@@ -636,27 +653,30 @@
         <v>6.1</v>
       </c>
       <c r="C6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D6" t="n">
         <v>1.6</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>0.8</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.7</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>4.6</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>5.2</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>2.1</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>9</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>5.6</v>
       </c>
     </row>
@@ -670,27 +690,30 @@
         <v>6.3</v>
       </c>
       <c r="C7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D7" t="n">
         <v>1.6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.8</v>
       </c>
       <c r="E7" t="n">
         <v>0.8</v>
       </c>
       <c r="F7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G7" t="n">
         <v>4.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>5.4</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>2.2</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>9</v>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>5.4</v>
       </c>
     </row>
@@ -704,27 +727,30 @@
         <v>6.2</v>
       </c>
       <c r="C8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D8" t="n">
         <v>1.6</v>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
         <v>0.8</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>0.7</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>4.6</v>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>5.3</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>2.1</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>9</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>5.6</v>
       </c>
     </row>

</xml_diff>